<commit_message>
video-seo-2026-09-25: fill traffic columns for 41 small sites from the Ahrefs Traffic panel
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/batches/2026-09-25-video-seo/14_video_seo_company_data.xlsx
+++ b/batches/2026-09-25-video-seo/14_video_seo_company_data.xlsx
@@ -4813,10 +4813,18 @@
       <c r="I91" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="J91" s="3" t="n"/>
-      <c r="K91" s="4" t="n"/>
-      <c r="L91" s="5" t="n"/>
-      <c r="M91" s="6" t="n"/>
+      <c r="J91" s="3" t="n">
+        <v>896</v>
+      </c>
+      <c r="K91" s="4" t="n">
+        <v>0.391</v>
+      </c>
+      <c r="L91" s="5" t="n">
+        <v>0.006064814814814815</v>
+      </c>
+      <c r="M91" s="6" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -6454,10 +6462,18 @@
       <c r="I126" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="J126" s="3" t="n"/>
-      <c r="K126" s="4" t="n"/>
-      <c r="L126" s="5" t="n"/>
-      <c r="M126" s="6" t="n"/>
+      <c r="J126" s="3" t="n">
+        <v>170</v>
+      </c>
+      <c r="K126" s="4" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="L126" s="5" t="n">
+        <v>0.00193287037037037</v>
+      </c>
+      <c r="M126" s="6" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -6634,10 +6650,18 @@
       <c r="I130" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="J130" s="3" t="n"/>
-      <c r="K130" s="4" t="n"/>
-      <c r="L130" s="5" t="n"/>
-      <c r="M130" s="6" t="n"/>
+      <c r="J130" s="3" t="n">
+        <v>234</v>
+      </c>
+      <c r="K130" s="4" t="n">
+        <v>0.905</v>
+      </c>
+      <c r="L130" s="5" t="n">
+        <v>0.000150462962962963</v>
+      </c>
+      <c r="M130" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6720,10 +6744,18 @@
       <c r="I132" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J132" s="3" t="n"/>
-      <c r="K132" s="4" t="n"/>
-      <c r="L132" s="5" t="n"/>
-      <c r="M132" s="6" t="n"/>
+      <c r="J132" s="3" t="n">
+        <v>129</v>
+      </c>
+      <c r="K132" s="4" t="n">
+        <v>0.655</v>
+      </c>
+      <c r="L132" s="5" t="n">
+        <v>0.0003703703703703704</v>
+      </c>
+      <c r="M132" s="6" t="n">
+        <v>1.1</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6759,10 +6791,18 @@
       <c r="I133" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J133" s="3" t="n"/>
-      <c r="K133" s="4" t="n"/>
-      <c r="L133" s="5" t="n"/>
-      <c r="M133" s="6" t="n"/>
+      <c r="J133" s="3" t="n">
+        <v>213</v>
+      </c>
+      <c r="K133" s="4" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L133" s="5" t="n">
+        <v>0.0001041666666666667</v>
+      </c>
+      <c r="M133" s="6" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -11423,10 +11463,18 @@
       <c r="I88" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J88" s="3" t="n"/>
-      <c r="K88" s="4" t="n"/>
-      <c r="L88" s="5" t="n"/>
-      <c r="M88" s="6" t="n"/>
+      <c r="J88" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="K88" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L88" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M88"/>
@@ -24621,10 +24669,18 @@
       <c r="I300" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J300" s="3" t="n"/>
-      <c r="K300" s="4" t="n"/>
-      <c r="L300" s="5" t="n"/>
-      <c r="M300" s="6" t="n"/>
+      <c r="J300" s="3" t="n">
+        <v>18700</v>
+      </c>
+      <c r="K300" s="4" t="n">
+        <v>0.436</v>
+      </c>
+      <c r="L300" s="5" t="n">
+        <v>0.00542824074074074</v>
+      </c>
+      <c r="M300" s="6" t="n">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -30560,10 +30616,18 @@
       <c r="I437" s="3" t="n">
         <v>9360</v>
       </c>
-      <c r="J437" s="3" t="n"/>
-      <c r="K437" s="4" t="n"/>
-      <c r="L437" s="5" t="n"/>
-      <c r="M437" s="6" t="n"/>
+      <c r="J437" s="3" t="n">
+        <v>587</v>
+      </c>
+      <c r="K437" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L437" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M437" s="6" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -37718,10 +37782,18 @@
       <c r="I603" s="3" t="n">
         <v>50</v>
       </c>
-      <c r="J603" s="3" t="n"/>
-      <c r="K603" s="4" t="n"/>
-      <c r="L603" s="5" t="n"/>
-      <c r="M603" s="6" t="n"/>
+      <c r="J603" s="3" t="n">
+        <v>330</v>
+      </c>
+      <c r="K603" s="4" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="L603" s="5" t="n">
+        <v>0.0001967592592592593</v>
+      </c>
+      <c r="M603" s="6" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="604">
       <c r="A604" t="inlineStr">
@@ -40173,10 +40245,18 @@
       <c r="I660" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J660" s="3" t="n"/>
-      <c r="K660" s="4" t="n"/>
-      <c r="L660" s="5" t="n"/>
-      <c r="M660" s="6" t="n"/>
+      <c r="J660" s="3" t="n">
+        <v>3800</v>
+      </c>
+      <c r="K660" s="4" t="n">
+        <v>0.416</v>
+      </c>
+      <c r="L660" s="5" t="n">
+        <v>0.002650462962962963</v>
+      </c>
+      <c r="M660" s="6" t="n">
+        <v>3.1</v>
+      </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
@@ -40724,10 +40804,18 @@
       <c r="I673" s="3" t="n">
         <v>56</v>
       </c>
-      <c r="J673" s="3" t="n"/>
-      <c r="K673" s="4" t="n"/>
-      <c r="L673" s="5" t="n"/>
-      <c r="M673" s="6" t="n"/>
+      <c r="J673" s="3" t="n">
+        <v>336</v>
+      </c>
+      <c r="K673" s="4" t="n">
+        <v>0.868</v>
+      </c>
+      <c r="L673" s="5" t="n">
+        <v>4.629629629629629e-05</v>
+      </c>
+      <c r="M673" s="6" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="674">
       <c r="A674" t="inlineStr">
@@ -41103,10 +41191,18 @@
       <c r="I682" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J682" s="3" t="n"/>
-      <c r="K682" s="4" t="n"/>
-      <c r="L682" s="5" t="n"/>
-      <c r="M682" s="6" t="n"/>
+      <c r="J682" s="3" t="n">
+        <v>143</v>
+      </c>
+      <c r="K682" s="4" t="n">
+        <v>0.745</v>
+      </c>
+      <c r="L682" s="5" t="n">
+        <v>0.005439814814814815</v>
+      </c>
+      <c r="M682" s="6" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="683">
       <c r="A683" t="inlineStr">
@@ -41349,10 +41445,18 @@
       <c r="I688" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J688" s="3" t="n"/>
-      <c r="K688" s="4" t="n"/>
-      <c r="L688" s="5" t="n"/>
-      <c r="M688" s="6" t="n"/>
+      <c r="J688" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="K688" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L688" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M688" s="6" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="689">
       <c r="A689" t="inlineStr">
@@ -41771,10 +41875,18 @@
       <c r="I698" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="J698" s="3" t="n"/>
-      <c r="K698" s="4" t="n"/>
-      <c r="L698" s="5" t="n"/>
-      <c r="M698" s="6" t="n"/>
+      <c r="J698" s="3" t="n">
+        <v>392</v>
+      </c>
+      <c r="K698" s="4" t="n">
+        <v>0.311</v>
+      </c>
+      <c r="L698" s="5" t="n">
+        <v>0.010625</v>
+      </c>
+      <c r="M698" s="6" t="n">
+        <v>1.9</v>
+      </c>
     </row>
     <row r="699">
       <c r="A699" t="inlineStr">
@@ -41806,10 +41918,18 @@
       <c r="I699" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J699" s="3" t="n"/>
-      <c r="K699" s="4" t="n"/>
-      <c r="L699" s="5" t="n"/>
-      <c r="M699" s="6" t="n"/>
+      <c r="J699" s="3" t="n">
+        <v>320</v>
+      </c>
+      <c r="K699" s="4" t="n">
+        <v>0.721</v>
+      </c>
+      <c r="L699" s="5" t="n">
+        <v>0.0001273148148148148</v>
+      </c>
+      <c r="M699" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="700">
       <c r="A700" t="inlineStr">
@@ -42271,10 +42391,18 @@
       <c r="I710" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J710" s="3" t="n"/>
-      <c r="K710" s="4" t="n"/>
-      <c r="L710" s="5" t="n"/>
-      <c r="M710" s="6" t="n"/>
+      <c r="J710" s="3" t="n">
+        <v>1700</v>
+      </c>
+      <c r="K710" s="4" t="n">
+        <v>0.697</v>
+      </c>
+      <c r="L710" s="5" t="n">
+        <v>0.002465277777777778</v>
+      </c>
+      <c r="M710" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="711">
       <c r="A711" t="inlineStr">
@@ -42478,10 +42606,18 @@
       <c r="I715" s="3" t="n">
         <v>37</v>
       </c>
-      <c r="J715" s="3" t="n"/>
-      <c r="K715" s="4" t="n"/>
-      <c r="L715" s="5" t="n"/>
-      <c r="M715" s="6" t="n"/>
+      <c r="J715" s="3" t="n">
+        <v>706</v>
+      </c>
+      <c r="K715" s="4" t="n">
+        <v>0.756</v>
+      </c>
+      <c r="L715" s="5" t="n">
+        <v>0.001770833333333333</v>
+      </c>
+      <c r="M715" s="6" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="716">
       <c r="A716" t="inlineStr">
@@ -42861,10 +42997,18 @@
       <c r="I724" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J724" s="3" t="n"/>
-      <c r="K724" s="4" t="n"/>
-      <c r="L724" s="5" t="n"/>
-      <c r="M724" s="6" t="n"/>
+      <c r="J724" s="3" t="n">
+        <v>1700</v>
+      </c>
+      <c r="K724" s="4" t="n">
+        <v>0.635</v>
+      </c>
+      <c r="L724" s="5" t="n">
+        <v>0.003298611111111111</v>
+      </c>
+      <c r="M724" s="6" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="725">
       <c r="A725" t="inlineStr">
@@ -43236,10 +43380,18 @@
       <c r="I733" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="J733" s="3" t="n"/>
-      <c r="K733" s="4" t="n"/>
-      <c r="L733" s="5" t="n"/>
-      <c r="M733" s="6" t="n"/>
+      <c r="J733" s="3" t="n">
+        <v>258</v>
+      </c>
+      <c r="K733" s="4" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="L733" s="5" t="n">
+        <v>0.0005092592592592592</v>
+      </c>
+      <c r="M733" s="6" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="734">
       <c r="A734" t="inlineStr">
@@ -43529,10 +43681,18 @@
       <c r="I740" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J740" s="3" t="n"/>
-      <c r="K740" s="4" t="n"/>
-      <c r="L740" s="5" t="n"/>
-      <c r="M740" s="6" t="n"/>
+      <c r="J740" s="3" t="n">
+        <v>550</v>
+      </c>
+      <c r="K740" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="L740" s="5" t="n">
+        <v>0.004722222222222222</v>
+      </c>
+      <c r="M740" s="6" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="741">
       <c r="A741" t="inlineStr">
@@ -43607,10 +43767,18 @@
       <c r="I742" s="3" t="n">
         <v>54</v>
       </c>
-      <c r="J742" s="3" t="n"/>
-      <c r="K742" s="4" t="n"/>
-      <c r="L742" s="5" t="n"/>
-      <c r="M742" s="6" t="n"/>
+      <c r="J742" s="3" t="n">
+        <v>285</v>
+      </c>
+      <c r="K742" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L742" s="5" t="n">
+        <v>0.001770833333333333</v>
+      </c>
+      <c r="M742" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="743">
       <c r="A743" t="inlineStr">
@@ -44115,10 +44283,18 @@
       <c r="I754" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="J754" s="3" t="n"/>
-      <c r="K754" s="4" t="n"/>
-      <c r="L754" s="5" t="n"/>
-      <c r="M754" s="6" t="n"/>
+      <c r="J754" s="3" t="n">
+        <v>139</v>
+      </c>
+      <c r="K754" s="4" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="L754" s="5" t="n">
+        <v>0.0003935185185185185</v>
+      </c>
+      <c r="M754" s="6" t="n">
+        <v>0.9</v>
+      </c>
     </row>
     <row r="755">
       <c r="A755" t="inlineStr">
@@ -44236,10 +44412,18 @@
       <c r="I757" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="J757" s="3" t="n"/>
-      <c r="K757" s="4" t="n"/>
-      <c r="L757" s="5" t="n"/>
-      <c r="M757" s="6" t="n"/>
+      <c r="J757" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="K757" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L757" s="5" t="n">
+        <v>0.01041666666666667</v>
+      </c>
+      <c r="M757" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="758">
       <c r="A758" t="inlineStr">
@@ -44486,10 +44670,18 @@
       <c r="I763" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J763" s="3" t="n"/>
-      <c r="K763" s="4" t="n"/>
-      <c r="L763" s="5" t="n"/>
-      <c r="M763" s="6" t="n"/>
+      <c r="J763" s="3" t="n">
+        <v>465</v>
+      </c>
+      <c r="K763" s="4" t="n">
+        <v>0.658</v>
+      </c>
+      <c r="L763" s="5" t="n">
+        <v>0.003043981481481481</v>
+      </c>
+      <c r="M763" s="6" t="n">
+        <v>2.1</v>
+      </c>
     </row>
     <row r="764">
       <c r="A764" t="inlineStr">
@@ -44607,10 +44799,18 @@
       <c r="I766" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="J766" s="3" t="n"/>
-      <c r="K766" s="4" t="n"/>
-      <c r="L766" s="5" t="n"/>
-      <c r="M766" s="6" t="n"/>
+      <c r="J766" s="3" t="n">
+        <v>502</v>
+      </c>
+      <c r="K766" s="4" t="n">
+        <v>0.789</v>
+      </c>
+      <c r="L766" s="5" t="n">
+        <v>0.00119212962962963</v>
+      </c>
+      <c r="M766" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="767">
       <c r="A767" t="inlineStr">
@@ -44685,10 +44885,18 @@
       <c r="I768" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J768" s="3" t="n"/>
-      <c r="K768" s="4" t="n"/>
-      <c r="L768" s="5" t="n"/>
-      <c r="M768" s="6" t="n"/>
+      <c r="J768" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="K768" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L768" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M768" s="6" t="n">
+        <v>0.7</v>
+      </c>
     </row>
     <row r="769">
       <c r="A769" t="inlineStr">
@@ -44720,10 +44928,18 @@
       <c r="I769" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J769" s="3" t="n"/>
-      <c r="K769" s="4" t="n"/>
-      <c r="L769" s="5" t="n"/>
-      <c r="M769" s="6" t="n"/>
+      <c r="J769" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="K769" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L769" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M769" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="770">
       <c r="A770" t="inlineStr">
@@ -44927,10 +45143,18 @@
       <c r="I774" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J774" s="3" t="n"/>
-      <c r="K774" s="4" t="n"/>
-      <c r="L774" s="5" t="n"/>
-      <c r="M774" s="6" t="n"/>
+      <c r="J774" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="K774" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L774" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M774" s="6" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="775">
       <c r="A775" t="inlineStr">
@@ -44962,10 +45186,18 @@
       <c r="I775" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J775" s="3" t="n"/>
-      <c r="K775" s="4" t="n"/>
-      <c r="L775" s="5" t="n"/>
-      <c r="M775" s="6" t="n"/>
+      <c r="J775" s="3" t="n">
+        <v>926</v>
+      </c>
+      <c r="K775" s="4" t="n">
+        <v>0.322</v>
+      </c>
+      <c r="L775" s="5" t="n">
+        <v>0.002905092592592593</v>
+      </c>
+      <c r="M775" s="6" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="776">
       <c r="A776" t="inlineStr">
@@ -45040,10 +45272,18 @@
       <c r="I777" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J777" s="3" t="n"/>
-      <c r="K777" s="4" t="n"/>
-      <c r="L777" s="5" t="n"/>
-      <c r="M777" s="6" t="n"/>
+      <c r="J777" s="3" t="n">
+        <v>276</v>
+      </c>
+      <c r="K777" s="4" t="n">
+        <v>0.633</v>
+      </c>
+      <c r="L777" s="5" t="n">
+        <v>0.001006944444444444</v>
+      </c>
+      <c r="M777" s="6" t="n">
+        <v>1.6</v>
+      </c>
     </row>
     <row r="778">
       <c r="A778" t="inlineStr">
@@ -45075,10 +45315,18 @@
       <c r="I778" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J778" s="3" t="n"/>
-      <c r="K778" s="4" t="n"/>
-      <c r="L778" s="5" t="n"/>
-      <c r="M778" s="6" t="n"/>
+      <c r="J778" s="3" t="n">
+        <v>65</v>
+      </c>
+      <c r="K778" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L778" s="5" t="n">
+        <v>0.009108796296296297</v>
+      </c>
+      <c r="M778" s="6" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="779">
       <c r="A779" t="inlineStr">
@@ -45110,10 +45358,18 @@
       <c r="I779" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J779" s="3" t="n"/>
-      <c r="K779" s="4" t="n"/>
-      <c r="L779" s="5" t="n"/>
-      <c r="M779" s="6" t="n"/>
+      <c r="J779" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="K779" s="4" t="n">
+        <v>0.308</v>
+      </c>
+      <c r="L779" s="5" t="n">
+        <v>0.0006712962962962962</v>
+      </c>
+      <c r="M779" s="6" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="780">
       <c r="A780" t="inlineStr">
@@ -45231,10 +45487,18 @@
       <c r="I782" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J782" s="3" t="n"/>
-      <c r="K782" s="4" t="n"/>
-      <c r="L782" s="5" t="n"/>
-      <c r="M782" s="6" t="n"/>
+      <c r="J782" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="K782" s="4" t="n">
+        <v>0.708</v>
+      </c>
+      <c r="L782" s="5" t="n">
+        <v>2.314814814814815e-05</v>
+      </c>
+      <c r="M782" s="6" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="783">
       <c r="A783" t="inlineStr">
@@ -45270,10 +45534,18 @@
       <c r="I783" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="J783" s="3" t="n"/>
-      <c r="K783" s="4" t="n"/>
-      <c r="L783" s="5" t="n"/>
-      <c r="M783" s="6" t="n"/>
+      <c r="J783" s="3" t="n">
+        <v>273</v>
+      </c>
+      <c r="K783" s="4" t="n">
+        <v>0.637</v>
+      </c>
+      <c r="L783" s="5" t="n">
+        <v>0.0003472222222222222</v>
+      </c>
+      <c r="M783" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="784">
       <c r="A784" t="inlineStr">
@@ -45348,10 +45620,18 @@
       <c r="I785" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J785" s="3" t="n"/>
-      <c r="K785" s="4" t="n"/>
-      <c r="L785" s="5" t="n"/>
-      <c r="M785" s="6" t="n"/>
+      <c r="J785" s="3" t="n">
+        <v>257</v>
+      </c>
+      <c r="K785" s="4" t="n">
+        <v>0.037</v>
+      </c>
+      <c r="L785" s="5" t="n">
+        <v>0.001319444444444444</v>
+      </c>
+      <c r="M785" s="6" t="n">
+        <v>1.7</v>
+      </c>
     </row>
     <row r="786">
       <c r="A786" t="inlineStr">
@@ -45641,10 +45921,18 @@
       <c r="I792" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J792" s="3" t="n"/>
-      <c r="K792" s="4" t="n"/>
-      <c r="L792" s="5" t="n"/>
-      <c r="M792" s="6" t="n"/>
+      <c r="J792" s="3" t="n">
+        <v>278</v>
+      </c>
+      <c r="K792" s="4" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="L792" s="5" t="n">
+        <v>0.001261574074074074</v>
+      </c>
+      <c r="M792" s="6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="793">
       <c r="A793" t="inlineStr">
@@ -45719,10 +46007,18 @@
       <c r="I794" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="J794" s="3" t="n"/>
-      <c r="K794" s="4" t="n"/>
-      <c r="L794" s="5" t="n"/>
-      <c r="M794" s="6" t="n"/>
+      <c r="J794" s="3" t="n">
+        <v>362</v>
+      </c>
+      <c r="K794" s="4" t="n">
+        <v>0.987</v>
+      </c>
+      <c r="L794" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M794" s="6" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="795">
       <c r="A795" t="inlineStr">
@@ -45797,10 +46093,18 @@
       <c r="I796" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J796" s="3" t="n"/>
-      <c r="K796" s="4" t="n"/>
-      <c r="L796" s="5" t="n"/>
-      <c r="M796" s="6" t="n"/>
+      <c r="J796" s="3" t="n">
+        <v>152</v>
+      </c>
+      <c r="K796" s="4" t="n">
+        <v>0.706</v>
+      </c>
+      <c r="L796" s="5" t="n">
+        <v>0.0003703703703703704</v>
+      </c>
+      <c r="M796" s="6" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="797">
       <c r="A797" t="inlineStr">
@@ -45832,10 +46136,18 @@
       <c r="I797" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J797" s="3" t="n"/>
-      <c r="K797" s="4" t="n"/>
-      <c r="L797" s="5" t="n"/>
-      <c r="M797" s="6" t="n"/>
+      <c r="J797" s="3" t="n">
+        <v>186</v>
+      </c>
+      <c r="K797" s="4" t="n">
+        <v>0.611</v>
+      </c>
+      <c r="L797" s="5" t="n">
+        <v>0.0001157407407407407</v>
+      </c>
+      <c r="M797" s="6" t="n">
+        <v>1.1</v>
+      </c>
     </row>
     <row r="798">
       <c r="A798" t="inlineStr">
@@ -45867,10 +46179,18 @@
       <c r="I798" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J798" s="3" t="n"/>
-      <c r="K798" s="4" t="n"/>
-      <c r="L798" s="5" t="n"/>
-      <c r="M798" s="6" t="n"/>
+      <c r="J798" s="3" t="n">
+        <v>1900</v>
+      </c>
+      <c r="K798" s="4" t="n">
+        <v>0.506</v>
+      </c>
+      <c r="L798" s="5" t="n">
+        <v>0.006064814814814815</v>
+      </c>
+      <c r="M798" s="6" t="n">
+        <v>2.1</v>
+      </c>
     </row>
     <row r="799">
       <c r="A799" t="inlineStr">
@@ -45902,10 +46222,18 @@
       <c r="I799" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J799" s="3" t="n"/>
-      <c r="K799" s="4" t="n"/>
-      <c r="L799" s="5" t="n"/>
-      <c r="M799" s="6" t="n"/>
+      <c r="J799" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="K799" s="4" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="L799" s="5" t="n">
+        <v>0.0001273148148148148</v>
+      </c>
+      <c r="M799" s="6" t="n">
+        <v>1.3</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M799"/>

</xml_diff>